<commit_message>
docs: retests front (A05, A06 corrigées), mise à jour du rapport du lot 1
</commit_message>
<xml_diff>
--- a/docs/Plan_de_tests_Lot1_Complet.xlsx
+++ b/docs/Plan_de_tests_Lot1_Complet.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="577" uniqueCount="355">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="577" uniqueCount="354">
   <si>
     <t xml:space="preserve">Plan de tests – Lot 1 – Projet Skull M1S1</t>
   </si>
@@ -731,7 +731,7 @@
     <t xml:space="preserve">Message « Le mot de passe doit contenir au moins 6 caractères » affiché, compte non créé</t>
   </si>
   <si>
-    <t xml:space="preserve">capture : T38_front_mdp_court.png</t>
+    <t xml:space="preserve">capture : T38_front_mdp_court.png. Retest 29/10/2026 après corrections du front : OK. Capture : T38_front_mdp_court_retest.png</t>
   </si>
   <si>
     <t xml:space="preserve">T39</t>
@@ -746,10 +746,10 @@
     <t xml:space="preserve">Messages sur les champs obligatoires</t>
   </si>
   <si>
-    <t xml:space="preserve">Un message sous chaque champ : « Le pseudo est obligatoire », « L'email est obligatoire », « Le mot de passe est obligatoire », « Confirme ton mot de passe ». Deux messages cumulés sous le mot de passe.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">capture : T39_front_champs_vides.png. Détail : doublon de messages sous le mot de passe (anomalie A05, issue #20).</t>
+    <t xml:space="preserve">Un message sous chaque champ obligatoire (pseudo, email, mot de passe, confirmation). Un seul message sous le mot de passe : « Le mot de passe est obligatoire ».</t>
+  </si>
+  <si>
+    <t xml:space="preserve">capture : T39_front_champs_vides.png (avant correction, doublon). Retest 29/10/2026 : doublon corrigé (anomalie A05, issue #20). Capture : T39_front_champs_vides_retest.png</t>
   </si>
   <si>
     <t xml:space="preserve">T40</t>
@@ -905,10 +905,10 @@
     <t xml:space="preserve">Le tableau de bord ne se réaffiche pas</t>
   </si>
   <si>
-    <t xml:space="preserve">Après la déconnexion, le bouton « Précédent » de Safari réaffiche temporairement le Dashboard du compte. Lors d’une interaction avec la page, redirection vers la page de connexion.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">capture : T48_front_retour_arriere.png. Voir anomalie A06 (issue #21).</t>
+    <t xml:space="preserve">Après la déconnexion, le bouton « Précédent » de Safari affiche la page de connexion ; le tableau de bord ne réapparaît plus.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">capture : T48_front_retour_arriere.png (avant correction, le tableau de bord réapparaissait). Retest 29/10/2026 : corrigé (anomalie A06, issue #21). Capture : T48_front_retour_arriere_retest.png</t>
   </si>
   <si>
     <t xml:space="preserve">T49</t>
@@ -1070,7 +1070,7 @@
     <t xml:space="preserve">A05</t>
   </si>
   <si>
-    <t xml:space="preserve">Page d'inscription, formulaire vide : deux messages s'affichent en même temps sous le champ mot de passe (« Le mot de passe doit contenir au moins 6 caractères » et « Le mot de passe est obligatoire »). Le premier est redondant quand le champ est vide.</t>
+    <t xml:space="preserve">Page d'inscription, formulaire vide : deux messages s'affichent en même temps sous le champ mot de passe (« Le mot de passe doit contenir au moins 6 caractères » et « Le mot de passe est obligatoire »). Le premier est redondant quand le champ est vide. Corrigé et retesté le 29/10/2026 (test T39).</t>
   </si>
   <si>
     <t xml:space="preserve">Front</t>
@@ -1079,13 +1079,10 @@
     <t xml:space="preserve">https://github.com/Rayanxdn/Skull_Game_M1S1/issues/20</t>
   </si>
   <si>
-    <t xml:space="preserve">Ouvert</t>
-  </si>
-  <si>
     <t xml:space="preserve">A06</t>
   </si>
   <si>
-    <t xml:space="preserve">Le tableau de bord réapparait avec le pseudo lors du retour en arrière après déconnexion</t>
+    <t xml:space="preserve">Le tableau de bord réapparait avec le pseudo lors du retour en arrière après déconnexion Corrigé et retesté le 29/10/2026 (test T48).</t>
   </si>
   <si>
     <t xml:space="preserve">https://github.com/Rayanxdn/Skull_Game_M1S1/issues/21</t>
@@ -1377,14 +1374,7 @@
     <cellStyle name="Currency [0]" xfId="18" builtinId="7"/>
     <cellStyle name="Percent" xfId="19" builtinId="5"/>
   </cellStyles>
-  <dxfs count="2">
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFFFFF"/>
-        </patternFill>
-      </fill>
-    </dxf>
+  <dxfs count="1">
     <dxf>
       <fill>
         <patternFill>
@@ -3598,7 +3588,7 @@
     <cfRule type="cellIs" priority="2" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="0">
       <formula>"OK"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="3" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="1">
+    <cfRule type="cellIs" priority="3" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="0">
       <formula>"Bloqué"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -4132,22 +4122,24 @@
         <v>350</v>
       </c>
       <c r="G7" s="22" t="s">
-        <v>351</v>
+        <v>335</v>
       </c>
       <c r="H7" s="24" t="n">
         <v>46324</v>
       </c>
-      <c r="I7" s="24"/>
+      <c r="I7" s="24" t="n">
+        <v>46324</v>
+      </c>
     </row>
     <row r="8" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="22" t="s">
-        <v>352</v>
+        <v>351</v>
       </c>
       <c r="B8" s="22" t="s">
         <v>289</v>
       </c>
       <c r="C8" s="22" t="s">
-        <v>353</v>
+        <v>352</v>
       </c>
       <c r="D8" s="22" t="s">
         <v>332</v>
@@ -4156,15 +4148,17 @@
         <v>349</v>
       </c>
       <c r="F8" s="23" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
       <c r="G8" s="22" t="s">
-        <v>351</v>
+        <v>335</v>
       </c>
       <c r="H8" s="24" t="n">
         <v>46324</v>
       </c>
-      <c r="I8" s="24"/>
+      <c r="I8" s="24" t="n">
+        <v>46324</v>
+      </c>
     </row>
     <row r="9" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="26"/>

</xml_diff>